<commit_message>
Ignora arquivos de dados e fotos
</commit_message>
<xml_diff>
--- a/LISTA DE OPERADORES.xlsx
+++ b/LISTA DE OPERADORES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\PROJETOS -BACKEND\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="S:\PROJETOS EM ANDAMENTO\PAINEL DE CONTROLE MTECH\PROGRAMAS\PROJETOS -BACKEND\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA0DCA52-6F81-45F7-9C5F-909FE62E276A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AA9D96B-B7AD-4627-82C0-AF52F011AA5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{AC9FE68F-77C9-4D03-9827-DD98DE9BB2CF}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{AC9FE68F-77C9-4D03-9827-DD98DE9BB2CF}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -39,47 +39,17 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
-  <si>
-    <t xml:space="preserve">JOSE LUCAS BAHIA              </t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>VANILDO ROCHA FRANCO</t>
   </si>
   <si>
-    <t xml:space="preserve">TIAGO SOUZA VICENTE           </t>
-  </si>
-  <si>
-    <t>EDNA TEIXEIRA</t>
-  </si>
-  <si>
-    <t>GESSÉ SEVERINO</t>
-  </si>
-  <si>
-    <t>GUILHERME</t>
-  </si>
-  <si>
-    <t>JONATHAN</t>
-  </si>
-  <si>
     <t>FRANCISCO FAUSTINO DA ROCHA</t>
   </si>
   <si>
-    <t>VALTERNEI MENDES</t>
-  </si>
-  <si>
-    <t>RAIMUNDO BARBOSA DOS SANTOS</t>
-  </si>
-  <si>
     <t>EDSON KERCHES</t>
   </si>
   <si>
-    <t>COSME DAMIÃO DOS SANTOS</t>
-  </si>
-  <si>
-    <t>JESIMOM JERIEL</t>
-  </si>
-  <si>
     <t>JULIO CESAR PELIZARI</t>
   </si>
   <si>
@@ -89,15 +59,9 @@
     <t>LIGIA DE MORAES</t>
   </si>
   <si>
-    <t>JEFERSON ANIZIO</t>
-  </si>
-  <si>
     <t>JOSE FAUSTINO</t>
   </si>
   <si>
-    <t>VALDIVINO DE SOUZA ROCHA</t>
-  </si>
-  <si>
     <t>EVANDRO PEREIRA DA SILVA</t>
   </si>
   <si>
@@ -110,25 +74,82 @@
     <t>FLAVIO MARCELO</t>
   </si>
   <si>
-    <t>CEZAR AUGUSTO DE SOUZA MAIA</t>
-  </si>
-  <si>
-    <t>MARCIO SILVA</t>
-  </si>
-  <si>
-    <t>CARLOS ANDRE</t>
-  </si>
-  <si>
-    <t>FABIO COSTA</t>
-  </si>
-  <si>
-    <t>GILBERTO SANTOS FERREIRA</t>
-  </si>
-  <si>
-    <t>ADSON SANTOS</t>
-  </si>
-  <si>
-    <t>FREDERICO ALVES</t>
+    <t>LUCIANO MALGUEIRO LIMA</t>
+  </si>
+  <si>
+    <t>CESAR AUGUSTO DE SOUZA MAIA</t>
+  </si>
+  <si>
+    <t>COSME DAMIÃO DOS SANTOS BATISTA</t>
+  </si>
+  <si>
+    <t>GESSE SEVERINO</t>
+  </si>
+  <si>
+    <t>JOSE LUCAS BAHIA</t>
+  </si>
+  <si>
+    <t>TIAGO SOUZA VICENTE</t>
+  </si>
+  <si>
+    <t>VALTERNEI MENDES DOS SANTOS</t>
+  </si>
+  <si>
+    <t>RAIMUNDO BARBOSA DOS SANTOS NE</t>
+  </si>
+  <si>
+    <t>JESIMOM JERIEL DE AQUINO</t>
+  </si>
+  <si>
+    <t>ALESSANDRA QUEIROZ</t>
+  </si>
+  <si>
+    <t>ROBERTO TADEU GERLACH</t>
+  </si>
+  <si>
+    <t>JOSE RICARDO ALBUQUERQUE</t>
+  </si>
+  <si>
+    <t>IVAN CARLOS</t>
+  </si>
+  <si>
+    <t>EDNA TEIXEIRA DA SILVA</t>
+  </si>
+  <si>
+    <t>PEDRO HENRIQUE</t>
+  </si>
+  <si>
+    <t>RAFAEL OLIVEIRA</t>
+  </si>
+  <si>
+    <t>SAMUEL SANDES</t>
+  </si>
+  <si>
+    <t>JONATHAN CORREIA</t>
+  </si>
+  <si>
+    <t>LUCAS TADEU ALMEIDA GERLACH</t>
+  </si>
+  <si>
+    <t>FREDERICO</t>
+  </si>
+  <si>
+    <t>MIQUÉIAS</t>
+  </si>
+  <si>
+    <t>RINALDO</t>
+  </si>
+  <si>
+    <t>ALAN</t>
+  </si>
+  <si>
+    <t>DIOGO</t>
+  </si>
+  <si>
+    <t>ALEX</t>
+  </si>
+  <si>
+    <t>HIAGO</t>
   </si>
 </sst>
 </file>
@@ -158,7 +179,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -181,20 +202,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -529,166 +556,201 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AA4E20E-2919-4396-A145-A937C26D729E}">
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="40.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
-        <v>23</v>
+      <c r="A3" s="1" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" s="4" t="s">
-        <v>11</v>
+      <c r="A4" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>3</v>
+      <c r="A5" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>10</v>
+      <c r="A6" s="1" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
-        <v>14</v>
+      <c r="A7" s="1" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>19</v>
+      <c r="A8" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>26</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>22</v>
+      <c r="A10" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>7</v>
+      <c r="A11" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>29</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" s="4" t="s">
-        <v>4</v>
+      <c r="A13" s="1" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>27</v>
+      <c r="A14" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>5</v>
+      <c r="A15" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
-        <v>16</v>
+      <c r="A16" s="1" t="s">
+        <v>23</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="4" t="s">
-        <v>12</v>
+      <c r="A17" s="1" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+      <c r="A18" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>0</v>
+      <c r="A20" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="4" t="s">
-        <v>13</v>
+      <c r="A21" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="4" t="s">
-        <v>15</v>
+      <c r="A22" s="1" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="3" t="s">
+      <c r="A24" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" s="4" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>1</v>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A30">
-    <sortCondition ref="A1:A30"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:A37">
+    <sortCondition ref="A1:A37"/>
   </sortState>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>